<commit_message>
- Bug fix .
</commit_message>
<xml_diff>
--- a/API_Trading/Calc.xlsx
+++ b/API_Trading/Calc.xlsx
@@ -544,37 +544,37 @@
         <v>0.39583333333333331</v>
       </c>
       <c r="B3">
-        <v>607.5</v>
+        <v>254.71</v>
       </c>
       <c r="C3">
-        <v>-10</v>
+        <v>-25</v>
       </c>
       <c r="D3">
         <f>B3*C3</f>
-        <v>-6075</v>
+        <v>-6367.75</v>
       </c>
       <c r="E3">
         <f>SUM(C3:C16)</f>
-        <v>-130</v>
+        <v>-35</v>
       </c>
       <c r="F3">
         <f>SUM(D3:D16)</f>
-        <v>-82459</v>
+        <v>-8937.75</v>
       </c>
       <c r="G3">
         <f>SUM(D3:D16)/E3</f>
-        <v>634.29999999999995</v>
+        <v>255.36428571428573</v>
       </c>
       <c r="H3">
-        <v>626.29999999999995</v>
+        <v>262</v>
       </c>
       <c r="I3">
         <f>((H3/$G$3)-1)*100</f>
-        <v>-1.2612328551158791</v>
+        <v>2.598528712483561</v>
       </c>
       <c r="J3">
         <f>$F$3*(I3/100)</f>
-        <v>1040.0000000000027</v>
+        <v>-232.24999999999946</v>
       </c>
       <c r="L3">
         <v>154.13</v>
@@ -648,25 +648,25 @@
         <v>10</v>
       </c>
       <c r="B4">
-        <v>625.6</v>
+        <v>257</v>
       </c>
       <c r="C4">
-        <v>-40</v>
+        <v>-10</v>
       </c>
       <c r="D4">
         <f t="shared" ref="D4:D16" si="0">B4*C4</f>
-        <v>-25024</v>
+        <v>-2570</v>
       </c>
       <c r="H4">
         <v>635</v>
       </c>
       <c r="I4">
         <f t="shared" ref="I4:I7" si="1">((H4/$G$3)-1)*100</f>
-        <v>0.11035787482265302</v>
+        <v>148.66437302453076</v>
       </c>
       <c r="J4">
         <f t="shared" ref="J4:J7" si="2">$F$3*(I4/100)</f>
-        <v>-91.000000000011454</v>
+        <v>-13287.249999999998</v>
       </c>
       <c r="L4">
         <v>151.01</v>
@@ -693,15 +693,9 @@
       <c r="A5" s="4">
         <v>0.4375</v>
       </c>
-      <c r="B5">
-        <v>642</v>
-      </c>
-      <c r="C5">
-        <v>-80</v>
-      </c>
       <c r="D5">
         <f t="shared" si="0"/>
-        <v>-51360</v>
+        <v>0</v>
       </c>
       <c r="I5">
         <f t="shared" si="1"/>
@@ -709,7 +703,7 @@
       </c>
       <c r="J5">
         <f t="shared" si="2"/>
-        <v>82459</v>
+        <v>8937.75</v>
       </c>
       <c r="L5">
         <v>150.07</v>
@@ -740,7 +734,7 @@
       </c>
       <c r="J6">
         <f t="shared" si="2"/>
-        <v>82459</v>
+        <v>8937.75</v>
       </c>
       <c r="N6">
         <f t="shared" si="3"/>
@@ -765,7 +759,7 @@
       </c>
       <c r="J7">
         <f t="shared" si="2"/>
-        <v>82459</v>
+        <v>8937.75</v>
       </c>
       <c r="N7">
         <f t="shared" si="3"/>

</xml_diff>